<commit_message>
Add cash allocation threshold research
</commit_message>
<xml_diff>
--- a/results/monthly_investor_report.xlsx
+++ b/results/monthly_investor_report.xlsx
@@ -15,12 +15,12 @@
     <sheet name="PAPER_TRADE" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'YONETICI_OZETI'!$A$6:$K$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PORTFOY_ONERISI'!$A$6:$O$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'YONETICI_OZETI'!$A$6:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PORTFOY_ONERISI'!$A$6:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ILK_20_SIRALAMA'!$A$1:$K$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AL_SAT_OZET'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AL_SAT_OZET'!$A$1:$B$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PIYASA_REJIMI'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PAPER_TRADE'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PAPER_TRADE'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -64,27 +64,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -129,55 +129,64 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -545,13 +554,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -668,16 +677,16 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.2183113574232514</v>
+        <v>0.1077292740640564</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>21831.13574232514</v>
+        <v>10772.92740640564</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.0573311795813907</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1251.60476370896</v>
+        <v>617.6246357539271</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>48.10856867095328</v>
@@ -688,7 +697,7 @@
       <c r="J7" s="4" t="n">
         <v>0.9590875530162508</v>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -709,16 +718,16 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.1869848989934444</v>
+        <v>0.09227072593594365</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>18698.48989934444</v>
+        <v>9227.072593594365</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>0.1135370331433445</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>2122.971067432362</v>
+        <v>1047.614446874969</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>94.87335182556761</v>
@@ -729,178 +738,49 @@
       <c r="J8" s="4" t="n">
         <v>2.270740662866885</v>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>BIMAS.IS</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>0.1725900803339808</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>17259.00803339808</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.0150053319741709</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>258.9771450860207</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>376.820729495411</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>352.6875</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>0.3001066394834209</v>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>TOASO.IS</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0.1648309264671155</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>16483.09264671155</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.035964069170425</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>592.7990840888577</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>306.6453644744458</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>277.2324952194509</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>0.5672232190119821</v>
-      </c>
-      <c r="K10" s="9" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>ARCLK.IS</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>0.1348305474093958</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>13483.05474093958</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.0318627708566734</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>429.6074836585416</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>107.313728169094</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0.6372554171334678</v>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>ASELS.IS</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>0.1224521893728121</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>12245.21893728121</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>0.0149130710450822</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>182.6138199742606</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>389.7266192813116</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>359.9101054961429</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>0.2377187363935803</v>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>CASH</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:K12"/>
+  <autoFilter ref="A6:K9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -911,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -941,7 +821,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Toplam önerilen/satılacak satır: 12</t>
+          <t>Toplam önerilen/satılacak satır: 13</t>
         </is>
       </c>
     </row>
@@ -1092,55 +972,55 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>SISE.IS</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="6" t="n">
         <v>45.5</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="5" t="n">
         <v>0.0063614591608023</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.0573311795813907</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="5" t="n">
         <v>0.1855133537025062</v>
       </c>
-      <c r="H8" s="14" t="n">
+      <c r="H8" s="6" t="n">
         <v>45.7894463918165</v>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="I8" s="6" t="n">
         <v>48.10856867095328</v>
       </c>
-      <c r="J8" s="14" t="n">
+      <c r="J8" s="6" t="n">
         <v>53.94085759346403</v>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="K8" s="6" t="n">
         <v>42.78015584943257</v>
       </c>
-      <c r="L8" s="13" t="n">
+      <c r="L8" s="4" t="n">
         <v>0.7970588235294117</v>
       </c>
-      <c r="M8" s="13" t="n">
+      <c r="M8" s="4" t="n">
         <v>64.34999999999999</v>
       </c>
-      <c r="N8" s="13" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>6A momentum pozitif; 3A momentum destekli; trend desteği var</t>
         </is>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Risk sinyali sınırlı</t>
         </is>
@@ -1157,7 +1037,7 @@
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="D9" s="14" t="n">
@@ -1212,7 +1092,7 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="D10" s="14" t="n">
@@ -1377,7 +1257,7 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="D13" s="14" t="n">
@@ -1422,55 +1302,55 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n">
+      <c r="A14" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>FROTO.IS</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="6" t="n">
         <v>85.19999694824219</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="5" t="n">
         <v>-0.0108077431499975</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="5" t="n">
         <v>0.1135370331433445</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="5" t="n">
         <v>0.1589867372070065</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="6" t="n">
         <v>84.27917726484502</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="I14" s="6" t="n">
         <v>94.87335182556761</v>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="J14" s="6" t="n">
         <v>98.74566647309014</v>
       </c>
-      <c r="K14" s="14" t="n">
+      <c r="K14" s="6" t="n">
         <v>80.93999710083007</v>
       </c>
-      <c r="L14" s="13" t="n">
+      <c r="L14" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="M14" s="13" t="n">
+      <c r="M14" s="4" t="n">
         <v>64.34999999999999</v>
       </c>
-      <c r="N14" s="13" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>hacim artışı var; volatilite görece düşük</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>kisa vadeli momentum negatif; trend desteği zayıf</t>
         </is>
@@ -1487,7 +1367,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">
@@ -1643,11 +1523,11 @@
     </row>
     <row r="18">
       <c r="A18" s="16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>YKBNK.IS</t>
+          <t>AKBNK.IS</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
@@ -1656,48 +1536,103 @@
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>33.41999816894531</v>
+        <v>63.70000076293945</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>-0.0659425781939114</v>
+        <v>-0.0615218226622063</v>
       </c>
       <c r="F18" s="18" t="n">
-        <v>-0.0310153372448183</v>
+        <v>-0.004687488079071</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.1010665940075984</v>
+        <v>0.1090908628521543</v>
       </c>
       <c r="H18" s="17" t="n">
-        <v>31.21619732644926</v>
+        <v>59.78106061241949</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>32.38346565501426</v>
+        <v>63.40140776872636</v>
       </c>
       <c r="J18" s="17" t="n">
-        <v>36.79764355562079</v>
+        <v>70.64908880985141</v>
       </c>
       <c r="K18" s="17" t="n">
-        <v>31.21619732644926</v>
+        <v>59.66295737853054</v>
       </c>
       <c r="L18" s="16" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4176470588235293</v>
       </c>
       <c r="M18" s="16" t="n">
         <v>64.34999999999999</v>
       </c>
       <c r="N18" s="16" t="inlineStr">
         <is>
+          <t>6A momentum pozitif; hacim artışı var</t>
+        </is>
+      </c>
+      <c r="O18" s="16" t="inlineStr">
+        <is>
+          <t>kisa vadeli momentum negatif; trend desteği zayıf; volatilite yüksek</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>YKBNK.IS</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>33.41999816894531</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>-0.0659425781939114</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>-0.0310153372448183</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>0.1010665940075984</v>
+      </c>
+      <c r="H19" s="17" t="n">
+        <v>31.21619732644926</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>32.38346565501426</v>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>36.79764355562079</v>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v>31.21619732644926</v>
+      </c>
+      <c r="L19" s="16" t="n">
+        <v>0.3764705882352941</v>
+      </c>
+      <c r="M19" s="16" t="n">
+        <v>64.34999999999999</v>
+      </c>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
           <t>Model skoru portföy için yeterli</t>
         </is>
       </c>
-      <c r="O18" s="16" t="inlineStr">
+      <c r="O19" s="16" t="inlineStr">
         <is>
           <t>kisa vadeli momentum negatif; trend desteği zayıf; volatilite yüksek</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:O18"/>
+  <autoFilter ref="A6:O19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1823,43 +1758,43 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>SISE.IS</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="4" t="n">
         <v>0.7970588235294117</v>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.0046066414674543</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.001115469846139</v>
       </c>
-      <c r="G3" s="15" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.235030926116428</v>
       </c>
-      <c r="H3" s="15" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.1566089169082498</v>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Kısmen trend üstü</t>
         </is>
       </c>
-      <c r="J3" s="15" t="n">
+      <c r="J3" s="5" t="n">
         <v>0.0298883972589827</v>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="5" t="n">
         <v>0.0573311795813907</v>
       </c>
     </row>
@@ -1877,7 +1812,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="E4" s="15" t="n">
@@ -1918,7 +1853,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="E5" s="15" t="n">
@@ -2041,7 +1976,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="E8" s="15" t="n">
@@ -2069,43 +2004,43 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>FROTO.IS</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="5" t="n">
         <v>-0.1310556420557422</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="5" t="n">
         <v>-0.2569639003843752</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="5" t="n">
         <v>-0.0072963800603302</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="5" t="n">
         <v>0.4702778794241973</v>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Trend altı</t>
         </is>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="5" t="n">
         <v>0.0232889396320691</v>
       </c>
-      <c r="K9" s="15" t="n">
+      <c r="K9" s="5" t="n">
         <v>0.1135370331433445</v>
       </c>
     </row>
@@ -2123,7 +2058,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TUT</t>
         </is>
       </c>
       <c r="E10" s="15" t="n">
@@ -2356,43 +2291,43 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n">
+      <c r="A16" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>AKBNK.IS</t>
         </is>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="16" t="n">
         <v>0.4176470588235293</v>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>PORTFOY_DISI</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="n">
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="n">
         <v>-0.1356851641707055</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="18" t="n">
         <v>-0.2830794788478351</v>
       </c>
-      <c r="G16" s="20" t="n">
+      <c r="G16" s="18" t="n">
         <v>0.0153144390476849</v>
       </c>
-      <c r="H16" s="20" t="n">
+      <c r="H16" s="18" t="n">
         <v>0.1238362901154654</v>
       </c>
-      <c r="I16" s="19" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <t>Trend altı</t>
         </is>
       </c>
-      <c r="J16" s="20" t="n">
+      <c r="J16" s="18" t="n">
         <v>0.0316879382736025</v>
       </c>
-      <c r="K16" s="20" t="n">
+      <c r="K16" s="18" t="n">
         <v>-0.004687488079071</v>
       </c>
     </row>
@@ -2490,7 +2425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2510,55 +2445,67 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Alınacaklar</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>SISE.IS, BIMAS.IS, TOASO.IS, ASELS.IS, FROTO.IS, ARCLK.IS</t>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>SISE.IS, FROTO.IS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Tutulacaklar</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>BIMAS.IS, TOASO.IS, ASELS.IS, ARCLK.IS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Satılacaklar</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>EREGL.IS, TCELL.IS, PETKM.IS, THYAO.IS, SAHOL.IS, YKBNK.IS</t>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>EREGL.IS, TCELL.IS, PETKM.IS, THYAO.IS, SAHOL.IS, AKBNK.IS, YKBNK.IS</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Portföy dışı kalanlar</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>KCHOL.IS, GARAN.IS, TUPRS.IS, AKBNK.IS, PGSUS.IS</t>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>KCHOL.IS, GARAN.IS, TUPRS.IS, PGSUS.IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Nakit kuralı</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Beklenen getiri %5 altında ise AL önerisi verilmez; kalan sermaye CASH olur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2589,66 +2536,66 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>BIST100 Güncel Kapanış</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="21" t="n">
         <v>13704</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>BIST100 MA200</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="21" t="n">
         <v>12248.34019042969</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Risk ON / Risk OFF</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Risk ON</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Aktif Model</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>volume_heavy</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Güven Puanı</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="21" t="n">
         <v>64.34999999999999</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Açıklama</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>BIST100 MA200 üzerinde olduğu için risk alma rejimi aktif.</t>
         </is>
@@ -2666,7 +2613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2722,307 +2669,277 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>PGSUS.IS</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2" s="22" t="n">
         <v>168.3999938964844</v>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="22" t="n">
         <v>168.3999938964844</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F2" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H2" s="5" t="n">
+      <c r="G2" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H2" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>AKBNK.IS</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>TUPRS.IS</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>63.70000076293945</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>63.70000076293945</v>
-      </c>
-      <c r="E3" s="5" t="n">
+      <c r="C3" s="22" t="n">
+        <v>244.8999938964844</v>
+      </c>
+      <c r="D3" s="22" t="n">
+        <v>244.8999938964844</v>
+      </c>
+      <c r="E3" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H3" s="5" t="n">
+      <c r="G3" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H3" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TUPRS.IS</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>GARAN.IS</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>244.8999938964844</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>244.8999938964844</v>
-      </c>
-      <c r="E4" s="5" t="n">
+      <c r="C4" s="22" t="n">
+        <v>123.0999984741211</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>123.0999984741211</v>
+      </c>
+      <c r="E4" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H4" s="5" t="n">
+      <c r="G4" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H4" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>GARAN.IS</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>ARCLK.IS</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
-        <v>123.0999984741211</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>123.0999984741211</v>
-      </c>
-      <c r="E5" s="5" t="n">
+      <c r="C5" s="22" t="n">
+        <v>104</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>104</v>
+      </c>
+      <c r="E5" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H5" s="5" t="n">
+      <c r="G5" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H5" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>ARCLK.IS</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>FROTO.IS</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>104</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>104</v>
-      </c>
-      <c r="E6" s="5" t="n">
+      <c r="C6" s="22" t="n">
+        <v>85.19999694824219</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>85.19999694824219</v>
+      </c>
+      <c r="E6" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H6" s="5" t="n">
+      <c r="G6" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H6" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>FROTO.IS</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>SISE.IS</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>85.19999694824219</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>85.19999694824219</v>
-      </c>
-      <c r="E7" s="5" t="n">
+      <c r="C7" s="22" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="E7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H7" s="5" t="n">
+      <c r="G7" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H7" s="23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SISE.IS</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>BIMAS.IS</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="E8" s="5" t="n">
+      <c r="C8" s="22" t="n">
+        <v>371.25</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>371.25</v>
+      </c>
+      <c r="E8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="22" t="n">
+        <v>-3.637978807091713e-12</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H8" s="5" t="n">
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>TOASO.IS</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>296</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>296</v>
+      </c>
+      <c r="E9" s="23" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>BIMAS.IS</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="F9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>ASELS.IS</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>371.25</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>371.25</v>
-      </c>
-      <c r="E9" s="5" t="n">
+      <c r="C10" s="22" t="n">
+        <v>384</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>384</v>
+      </c>
+      <c r="E10" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="6" t="n">
-        <v>-3.637978807091713e-12</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H9" s="5" t="n">
+      <c r="F10" s="22" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>TOASO.IS</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>296</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>296</v>
-      </c>
-      <c r="E10" s="5" t="n">
+      <c r="G10" s="22" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H10" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>ASELS.IS</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>384</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>384</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>180000</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>